<commit_message>
table formats and terminology updated
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/doc/source/_static/data/supporting_files/Terminology.xlsx
+++ b/doc/source/_static/data/supporting_files/Terminology.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzorinaldi/Documents/GitHub/MARIO/doc/source/_static/data/supporting_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C34F573-4B2A-C444-A947-5D592C28D65C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0774540-8828-1541-9D53-BED721D08A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26880" activeTab="4" xr2:uid="{191C6CC1-D0C2-3B4B-A0D5-6A4A3794157A}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26880" activeTab="2" xr2:uid="{191C6CC1-D0C2-3B4B-A0D5-6A4A3794157A}"/>
   </bookViews>
   <sheets>
     <sheet name="Matrices" sheetId="1" r:id="rId1"/>

</xml_diff>